<commit_message>
Add V61 multi-site temporal reproducibility
</commit_message>
<xml_diff>
--- a/supplementary_data/Supplementary_Data_6_parametric_case_and_lc_erl_codebook.xlsx
+++ b/supplementary_data/Supplementary_Data_6_parametric_case_and_lc_erl_codebook.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lc_erl_codebook" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mini_audit_template" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provenance_notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="multisite_temporal_index" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_descriptors_multisite" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27561,13 +27563,6 @@
           <t>blind_record_01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27580,13 +27575,6 @@
           <t>blind_record_02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27599,13 +27587,6 @@
           <t>blind_record_03</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27618,13 +27599,6 @@
           <t>blind_record_04</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27637,13 +27611,6 @@
           <t>blind_record_05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27656,13 +27623,6 @@
           <t>blind_record_06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27675,13 +27635,6 @@
           <t>blind_record_07</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27694,13 +27647,6 @@
           <t>blind_record_08</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27713,13 +27659,6 @@
           <t>blind_record_09</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27732,13 +27671,6 @@
           <t>blind_record_10</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27751,13 +27683,6 @@
           <t>blind_record_11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27770,13 +27695,6 @@
           <t>blind_record_12</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27789,13 +27707,6 @@
           <t>blind_record_13</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27808,13 +27719,6 @@
           <t>blind_record_14</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27827,13 +27731,6 @@
           <t>blind_record_15</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27846,13 +27743,6 @@
           <t>blind_record_16</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27865,13 +27755,6 @@
           <t>blind_record_17</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27884,13 +27767,6 @@
           <t>blind_record_18</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27903,13 +27779,6 @@
           <t>blind_record_19</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27922,13 +27791,6 @@
           <t>blind_record_20</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27941,13 +27803,6 @@
           <t>blind_record_21</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27960,13 +27815,6 @@
           <t>blind_record_22</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27979,13 +27827,6 @@
           <t>blind_record_23</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -27998,13 +27839,6 @@
           <t>blind_record_24</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -28017,13 +27851,6 @@
           <t>blind_record_25</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>for independent non-author coder; no external agreement is claimed in the manuscript</t>
@@ -28091,4 +27918,669 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>longest_shadow_h</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>longest_shadow_d</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>height_above_ground</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>site_source</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>nominal_delivered_energy_MJ_per_kg</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>temporal_storage_sensitivity_MJ_d_per_kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Shackleton rim</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>66</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2 (65-66 h, two spots)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cold sinter</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>2.016806722689076</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5.546218487394959</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Shackleton rim</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>66</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2 (65-66 h, two spots)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>4.329004329004329</v>
+      </c>
+      <c r="H3" t="n">
+        <v>11.9047619047619</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Shackleton rim</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>66</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2 (65-66 h, two spots)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Geopolymer</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>4.563279857397505</v>
+      </c>
+      <c r="H4" t="n">
+        <v>12.54901960784314</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Shackleton rim</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2 (65-66 h, two spots)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>25.97402597402597</v>
+      </c>
+      <c r="H5" t="n">
+        <v>71.42857142857142</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>112</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cold sinter</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2.016806722689076</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9.411764705882357</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C1</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>112</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>4.329004329004329</v>
+      </c>
+      <c r="H7" t="n">
+        <v>20.2020202020202</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C1</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>112</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Geopolymer</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>4.563279857397505</v>
+      </c>
+      <c r="H8" t="n">
+        <v>21.29530600118836</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>112</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>25.97402597402597</v>
+      </c>
+      <c r="H9" t="n">
+        <v>121.2121212121212</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C2</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>165</v>
+      </c>
+      <c r="C10" t="n">
+        <v>6.875</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Cold sinter</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2.016806722689076</v>
+      </c>
+      <c r="H10" t="n">
+        <v>13.8655462184874</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C2</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>165</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6.875</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>4.329004329004329</v>
+      </c>
+      <c r="H11" t="n">
+        <v>29.76190476190476</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C2</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>165</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6.875</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Geopolymer</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>4.563279857397505</v>
+      </c>
+      <c r="H12" t="n">
+        <v>31.37254901960785</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Connecting Ridge C2</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>165</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6.875</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2 m</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Glaser2018_T2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>25.97402597402597</v>
+      </c>
+      <c r="H13" t="n">
+        <v>178.5714285714286</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Barker Site-1</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>192</v>
+      </c>
+      <c r="C14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>5 m</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Barker2021_high_LCSP (4-8 d; high case)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Cold sinter</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>2.016806722689076</v>
+      </c>
+      <c r="H14" t="n">
+        <v>16.13445378151261</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Barker Site-1</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>192</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>5 m</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Barker2021_high_LCSP (4-8 d; high case)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>4.329004329004329</v>
+      </c>
+      <c r="H15" t="n">
+        <v>34.63203463203463</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Barker Site-1</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>192</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5 m</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Barker2021_high_LCSP (4-8 d; high case)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Geopolymer</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>4.563279857397505</v>
+      </c>
+      <c r="H16" t="n">
+        <v>36.50623885918004</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Barker Site-1</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>192</v>
+      </c>
+      <c r="C17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>5 m</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Barker2021_high_LCSP (4-8 d; high case)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SPS</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>25.97402597402597</v>
+      </c>
+      <c r="H17" t="n">
+        <v>207.7922077922078</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_used</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Glaser et al. 2018 PSS / NTRS 20170007365</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Shackleton rim 66 h; Connecting Ridge C1 112 h; Connecting Ridge C2 165 h</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>published 20-year LOLA-DTM descriptors at 2 m; no new illumination modelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Barker/PGDA Site-1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>8 d high-case dark gap</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>published descriptor at 5 m; used for stress screen</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>